<commit_message>
How to Create Django Project
</commit_message>
<xml_diff>
--- a/02. ETC/26년_작업기록.xlsx
+++ b/02. ETC/26년_작업기록.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeon_\OneDrive\デスクトップ\__CODE__\02. ETC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5B9CB3-F859-4798-AC2B-28BEF7CC0A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{081CABCC-31C9-4EFC-BD28-45B629BC61A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4185" yWindow="2370" windowWidth="21600" windowHeight="11295" firstSheet="2" activeTab="6" xr2:uid="{3AB49DFB-F50B-4E0E-B2FE-464404D0CD6F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="6" xr2:uid="{3AB49DFB-F50B-4E0E-B2FE-464404D0CD6F}"/>
   </bookViews>
   <sheets>
     <sheet name="01. Git Command" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="140">
   <si>
     <t xml:space="preserve">1. 현재 브랜치 확인 시도 </t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -542,11 +542,58 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>1. 파이썬 설치 -&gt; 환경변수? 아직안함.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>2. Django 설치 -&gt; cmd에서 -&gt; py -m pip install Django==6.0.4</t>
+    <t># ================================================</t>
+  </si>
+  <si>
+    <t># 프로젝트 폴더: C:\Users\jeon_\OneDrive\데스크톱\ptsol-mobile-order-system\project</t>
+  </si>
+  <si>
+    <t># 1. VS Code 터미널을 PowerShell로 변경 (처음 1회)</t>
+  </si>
+  <si>
+    <t>#   → 하단 터미널에서 MINGW64 클릭 → Select Default Profile → PowerShell 선택</t>
+  </si>
+  <si>
+    <t># 2. 가상환경 생성 (처음 1회만 실행)</t>
+  </si>
+  <si>
+    <t>python -m venv venv</t>
+  </si>
+  <si>
+    <t># 3. 가상환경 활성화</t>
+  </si>
+  <si>
+    <t>venv\Scripts\activate</t>
+  </si>
+  <si>
+    <t># 4. Django 설치</t>
+  </si>
+  <si>
+    <t>pip install django</t>
+  </si>
+  <si>
+    <t># 5. Django 프로젝트 생성 (현재 폴더에 바로 생성)</t>
+  </si>
+  <si>
+    <t>django-admin startproject config .</t>
+  </si>
+  <si>
+    <t># 6. 개발 서버 실행</t>
+  </si>
+  <si>
+    <t>python manage.py runserver</t>
+  </si>
+  <si>
+    <t># 서버 접속 주소</t>
+  </si>
+  <si>
+    <t># http://127.0.0.1:8000</t>
+  </si>
+  <si>
+    <t># 서버 멈추기: Ctrl + C</t>
+  </si>
+  <si>
+    <t># Django 프로젝트 설정 전체 과정</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1775,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{090EC465-0E4C-4318-9D81-186DFF8FAE5D}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1783,9 +1830,99 @@
         <v>122</v>
       </c>
     </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>139</v>
+      </c>
+    </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>